<commit_message>
Fix truncation and ID_OBJECTIF errors in the SQL Server injection script
- POSTE codes now hard-capped at 12 chars (real varchar(12) limit) with
  safe dedup on truncation.
- CODE_COMPETENCE codes kept as-is (>8 chars like ACH-BO-009), paired
  with a new alter_code_competence.sql widening CODE_COMPETENCE and
  POSTE_CRITERES.CODE_COMPETENCE to varchar(20).
- ID_OBJECTIF (not an IDENTITY column) is now computed via a running
  @next_obj_id variable instead of being omitted (was causing a NOT
  NULL violation).
- All free-text fields are now truncated to their real varchar limits
  (DIMENSION 250, OBSERVATIONS 550, INTITULE 90, etc.) instead of
  risking a truncation error at execution; every truncation is logged
  in a new "Troncatures appliquées" sheet in the review workbook.
- Fixed DEGRE_MAITRISE extraction (was never populated due to a
  isdigit() check against "N4"-style strings instead of the digit).
</commit_message>
<xml_diff>
--- a/data/import_review.xlsx
+++ b/data/import_review.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NIVEAU_ETUDE non mappés" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CODE_COMPETENCE manquants" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compétences non matchées" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Troncatures appliquées" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -549,7 +550,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ACH_CHEF_EXPLOITATION_ACHATS</t>
+          <t>ACH_CHEF_EXP</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -626,7 +627,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ACH_DIRECTEUR_ACHAT_FERRAILL</t>
+          <t>ACH_DIRECTEU</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -660,7 +661,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ACH_DIRECTEUR_ADJOINT_CHARGE</t>
+          <t>ACH_DIRECTE2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -733,7 +734,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ACH_PURCHASING_DATA_MASTER</t>
+          <t>ACH_PURCHASI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -806,7 +807,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ACH_RESPONSABLE_ACHATS_CAPEX</t>
+          <t>ACH_RESPONSA</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -992,7 +993,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ACH_RESPONSABLE_MASTER_DATA</t>
+          <t>ACH_RESPONS2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1065,12 +1066,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ACH_FAC_001_2</t>
+          <t>ACH_FAC_0012</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -1143,7 +1144,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ACH_RESPONSABLE_FAMILLE_ACHA</t>
+          <t>ACH_RESPONS3</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1177,7 +1178,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ACH_RESPONSABLE_LOGISTIQUE_B</t>
+          <t>ACH_RESPONS4</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1211,12 +1212,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ACH_RCP_01_2</t>
+          <t>ACH_RCP_012</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1285,7 +1286,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>JUR_DIRECTEUR_JURIDIQUE_RISK</t>
+          <t>JUR_DIRECTEU</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1315,7 +1316,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>JUR_JURISTE_JUNIOR</t>
+          <t>JUR_JURISTE</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1380,7 +1381,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>JUR_RESPONSABLE_CONTROLE_INT</t>
+          <t>JUR_RESPONSA</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1410,7 +1411,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>JUR_RESPONSABLE_JURIDIQUE</t>
+          <t>JUR_RESPONS2</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1440,7 +1441,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>JUR_RESPONSABLE_RISK_MANAGEM</t>
+          <t>JUR_RESPONS3</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1470,7 +1471,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AUD_AUDITEUR_SENIOR</t>
+          <t>AUD_AUDITEUR</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1504,7 +1505,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>AUD_HEAD_OF_AUDIT</t>
+          <t>AUD_HEAD_OF</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1534,12 +1535,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>DIR_BD_EC_001</t>
+          <t>DIR_BD_EC_00</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -1639,12 +1640,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SON_IND_BPEC_2024</t>
+          <t>SON_IND_BPEC</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -1674,7 +1675,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DCM_CHARGE_ADMINITRATION_VEN</t>
+          <t>DCM_CHARGE_A</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1708,7 +1709,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>DCM_CHARGEE_RELATION_CLIENTS</t>
+          <t>DCM_CHARGEE</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1742,7 +1743,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>DCM_CHEF_EXP_MARKETING</t>
+          <t>DCM_CHEF_EXP</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1776,7 +1777,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>DCM_CHEF_EXPL_PERF</t>
+          <t>DCM_CHEF_EX2</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1810,7 +1811,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>DCM_CHEF_EXPLOITATION_CHARGE</t>
+          <t>DCM_CHEF_EX3</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1844,7 +1845,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>DCM_CHEF_PROJET_MARKETING</t>
+          <t>DCM_CHEF_PRO</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1878,7 +1879,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DCM_CHIEF_COMMERCIAL_MARKETI</t>
+          <t>DCM_CHIEF_CO</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1912,7 +1913,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>DCM_CUSTOMER_RELATIONSHIP_MA</t>
+          <t>DCM_CUSTOMER</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1946,7 +1947,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>DCM_DIRECTEUR_ADJOINT_CHARGE</t>
+          <t>DCM_DIRECTEU</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1980,7 +1981,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>DCM_DIRECTEUR_COMMERCIAL_ADJ</t>
+          <t>DCM_DIRECTE2</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2014,7 +2015,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>DCM_DIRECTEUR_VENTES</t>
+          <t>DCM_DIRECTE3</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2087,7 +2088,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>DCM_RESP_MARKETING_COMMUNICA</t>
+          <t>DCM_RESP_MAR</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2121,7 +2122,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>DCM_RESPONSABLE_RELATION_CLI</t>
+          <t>DCM_RESPONSA</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2155,7 +2156,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>DCM_RESPONSABLE_ADMINISTRATI</t>
+          <t>DCM_RESPONS2</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2189,7 +2190,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>DCM_RESPONSABLE_VENTES_REGIO</t>
+          <t>DCM_RESPONS3</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2262,7 +2263,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>DCM_SALES_OPTIMIZATION_MANAG</t>
+          <t>DCM_SALES_OP</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2296,7 +2297,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>DCM_TECHNICO_COMMERCIAL</t>
+          <t>DCM_TECHNICO</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2361,7 +2362,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>FIN_CHARGE_CREDIT_CLIENT</t>
+          <t>FIN_CHARGE_C</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2391,7 +2392,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>FIN_CHARGEE_TRESORERIE</t>
+          <t>FIN_CHARGEE</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2421,7 +2422,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>FIN_CHEF_COMPTABLE</t>
+          <t>FIN_CHEF_COM</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2451,7 +2452,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>FIN_CHEF_EXPLOITATION_CHARGE</t>
+          <t>FIN_CHEF_EXP</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2481,7 +2482,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>FIN_COMPTABLE_CLIENT</t>
+          <t>FIN_COMPTABL</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2511,7 +2512,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>FIN_COMPTABLE_FOURNISSEUR</t>
+          <t>FIN_COMPTAB2</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2576,7 +2577,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>FIN_DIR_ADJ_CONTROLLING</t>
+          <t>FIN_DIR_ADJ</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2606,7 +2607,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>FIN_DIRECTEUR_ADJOINT_CHARGE</t>
+          <t>FIN_DIRECTEU</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2636,7 +2637,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>FIN_DIRECTEUR_ADJOINT_CHARGE_2</t>
+          <t>FIN_DIRECTE2</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2666,7 +2667,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>FIN_DIRECTEUR_COMPTABILITE_C</t>
+          <t>FIN_DIRECTE3</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2696,7 +2697,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>FIN_INDUSTRIAL_CONTROLLER</t>
+          <t>FIN_INDUSTRI</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2726,7 +2727,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>FIN_JUNIOR_FINANCIAL_CONTROL</t>
+          <t>FIN_JUNIOR_F</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2756,7 +2757,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>FIN_RESPONSABLE_COMPTABILITE</t>
+          <t>FIN_RESPONSA</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2786,7 +2787,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>FIN_RESPONSABLE_COMPTABILITE_2</t>
+          <t>FIN_RESPONS2</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2816,7 +2817,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>FIN_RESPONSABLE_CREDIT_CLIEN</t>
+          <t>FIN_RESPONS3</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2846,7 +2847,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>FIN_RESPONSABLE_REPORTING_IF</t>
+          <t>FIN_RESPONS4</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2876,7 +2877,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>FIN_RESPOSABLE_COMPTABILITE</t>
+          <t>FIN_RESPOSAB</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2906,7 +2907,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>FIN_SENIOR_FINANCIAL_CONTROL</t>
+          <t>FIN_SENIOR_F</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2936,7 +2937,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>FIN_TRESORIER_CHARGE_REPORTI</t>
+          <t>FIN_TRESORIE</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2966,7 +2967,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>DG_CHIEF_STRATEGY_DIGITAL</t>
+          <t>DG_CHIEF_STR</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3039,12 +3040,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>DIR_BU_CUAL_2024</t>
+          <t>DIR_BU_CUAL_</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C78" t="inlineStr"/>
@@ -3144,12 +3145,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SST_MGR_IND_01</t>
+          <t>SST_MGR_IND_</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C81" t="inlineStr"/>
@@ -3179,12 +3180,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CE_PFBP_DI_001</t>
+          <t>CE_PFBP_DI_0</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C82" t="inlineStr"/>
@@ -3257,7 +3258,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>IND_CHEF_EXPLOITATION_ACIERI</t>
+          <t>IND_CHEF_EXP</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -3295,12 +3296,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>PROD_CHEF_EXPL_NAD</t>
+          <t>PROD_CHEF_EX</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C85" t="inlineStr"/>
@@ -3373,12 +3374,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>SON_DI_ADRH_024</t>
+          <t>SON_DI_ADRH_</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C87" t="inlineStr"/>
@@ -3451,12 +3452,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>DI_ADJ_TCO_001</t>
+          <t>DI_ADJ_TCO_0</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C89" t="inlineStr"/>
@@ -3490,12 +3491,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>DIR_MAINT_002</t>
+          <t>DIR_MAINT_00</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C90" t="inlineStr"/>
@@ -3529,12 +3530,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>DI_LAM_DIRADJ</t>
+          <t>DI_LAM_DIRAD</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C91" t="inlineStr"/>
@@ -3685,12 +3686,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>DIR_SITE_NAD_001</t>
+          <t>DIR_SITE_NAD</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C95" t="inlineStr"/>
@@ -3763,12 +3764,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ENG_MAINT_ACI</t>
+          <t>ENG_MAINT_AC</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C97" t="inlineStr"/>
@@ -3841,12 +3842,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ING_PROD_LAM_001</t>
+          <t>ING_PROD_LAM</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C99" t="inlineStr"/>
@@ -3919,12 +3920,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>IPP_TECH_2024</t>
+          <t>IPP_TECH_202</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C101" t="inlineStr"/>
@@ -3997,12 +3998,12 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>MAINT_CAPEX_001</t>
+          <t>MAINT_CAPEX_</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C103" t="inlineStr"/>
@@ -4075,12 +4076,12 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>MAINT_ELEC_ACI_001</t>
+          <t>MAINT_ELEC_A</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C105" t="inlineStr"/>
@@ -4114,12 +4115,12 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>MAINT_ELEC_LAM_2024</t>
+          <t>MAINT_ELEC_L</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C106" t="inlineStr"/>
@@ -4270,12 +4271,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>MAINT_METH_001</t>
+          <t>MAINT_METH_0</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C110" t="inlineStr"/>
@@ -4309,12 +4310,12 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>MAINT_FIAB_001</t>
+          <t>MAINT_FIAB_0</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C111" t="inlineStr"/>
@@ -4348,12 +4349,12 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>SC_MAG_NAD_01</t>
+          <t>SC_MAG_NAD_0</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C112" t="inlineStr"/>
@@ -4387,12 +4388,12 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>MAINT_MECA_NAD_001</t>
+          <t>MAINT_MECA_N</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C113" t="inlineStr"/>
@@ -4426,12 +4427,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>MNT_ELEC_NAD_001</t>
+          <t>MNT_ELEC_NAD</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C114" t="inlineStr"/>
@@ -4504,12 +4505,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>IND_PLAN_FER_001</t>
+          <t>IND_PLAN_FER</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C116" t="inlineStr"/>
@@ -4543,12 +4544,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>DI_PROD_FAC_01</t>
+          <t>DI_PROD_FAC_</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C117" t="inlineStr"/>
@@ -4621,7 +4622,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>IND_RESPONSABLE_PRODUCTION_C</t>
+          <t>IND_RESPONSA</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -4659,12 +4660,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>QUAL_RESP_001</t>
+          <t>QUAL_RESP_00</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C120" t="inlineStr"/>
@@ -4698,12 +4699,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>SC_MAG_NAD_01_2</t>
+          <t>SC_MAG_NAD_2</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
@@ -4737,12 +4738,12 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>MAINT_ELEC_001</t>
+          <t>MAINT_ELEC_0</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Code poste source</t>
+          <t>Code poste source (tronqué)</t>
         </is>
       </c>
       <c r="C122" t="inlineStr"/>
@@ -4815,7 +4816,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>STRAT_CHEF_EXPLOITATION_CHARGE</t>
+          <t>STRAT_CHEF_E</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -4849,7 +4850,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>STRAT_CHEF_PROJET_STRATEGIE</t>
+          <t>STRAT_CHEF_P</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -4953,7 +4954,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>GEN_AGENT_PONT_BASCULE</t>
+          <t>GEN_AGENT_PO</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -4987,7 +4988,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>GEN_CHARGE_TRANSPORT</t>
+          <t>GEN_CHARGE_T</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -5017,7 +5018,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>GEN_CHARGE_CONSIGNATION</t>
+          <t>GEN_CHARGE_C</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -5047,7 +5048,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>GEN_CHARGE_MOYENS_GENERAUX</t>
+          <t>GEN_CHARGE_M</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -5077,7 +5078,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>GEN_CONTROLEUR_EXPEDITEUR_PR</t>
+          <t>GEN_CONTROLE</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -5107,7 +5108,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>GEN_DIRECTRICE_ADJOINTE_CHAR</t>
+          <t>GEN_DIRECTRI</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -5141,7 +5142,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>GEN_EXPEDITEUR</t>
+          <t>GEN_EXPEDITE</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -5171,7 +5172,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>GEN_INGENIEUR_SST</t>
+          <t>GEN_INGENIEU</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -5201,7 +5202,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>GEN_MANUTENTIONNAIRE</t>
+          <t>GEN_MANUTENT</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -5235,7 +5236,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>GEN_PONTIER_EXPEDITION</t>
+          <t>GEN_PONTIER</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -5265,7 +5266,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>GEN_RESPONSABLE_DIGITALISATI</t>
+          <t>GEN_RESPONSA</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -5299,7 +5300,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>GEN_RESPONSABLE_OPERATIONS_L</t>
+          <t>GEN_RESPONS2</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -5329,7 +5330,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>GEN_RESPONSABLE_RECEPTION_FE</t>
+          <t>GEN_RESPONS3</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -5359,7 +5360,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>GEN_RESPONSABLE_SONASID_DIST</t>
+          <t>GEN_RESPONS4</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -5389,7 +5390,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>GEN_RESPONSABLE_TRANSPORT</t>
+          <t>GEN_RESPONS5</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -5419,7 +5420,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>GEN_RESPONSABLE_ACTIVITES_PO</t>
+          <t>GEN_RESPONS6</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -5449,7 +5450,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>GEN_SUPERVISEUR_RECEPTION_FE</t>
+          <t>GEN_SUPERVIS</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -5479,7 +5480,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>GEN_SUPERVISEUR_PONT_BASCULE</t>
+          <t>GEN_SUPERVI2</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -5509,7 +5510,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>GEN_SUPPLY_CHAIN_MANAGER</t>
+          <t>GEN_SUPPLY_C</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -5543,7 +5544,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>SI_DIRECTEUR_ADJOINT_CHARGE</t>
+          <t>SI_DIRECTEUR</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -5581,7 +5582,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>SI_IT_PROJECT_LEAD</t>
+          <t>SI_IT_PROJEC</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -5619,7 +5620,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>SI_IT_PROJECT_MANAGER</t>
+          <t>SI_IT_PROJE2</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -5657,7 +5658,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>SI_INFRASTRUCTURE_AND_SECUR</t>
+          <t>SI_INFRASTRU</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -5695,7 +5696,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>SI_INGENIEUR_ETUDES_DEVELOP</t>
+          <t>SI_INGENIEUR</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -5733,7 +5734,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>SI_RESPONSABLE_INFRASTRUCTU</t>
+          <t>SI_RESPONSAB</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -5771,7 +5772,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>SI_RESPONSABLE_SECURITE_SI</t>
+          <t>SI_RESPONSA2</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -5809,7 +5810,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>SI_TECHNICIEN_IT_SITE</t>
+          <t>SI_TECHNICIE</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -5843,7 +5844,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>TECH_CHEF_EXPLOITATION_PROJET</t>
+          <t>TECH_CHEF_EX</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -5877,7 +5878,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>TECH_DIRECTEUR_PERFORMANCE_IN</t>
+          <t>TECH_DIRECTE</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -5911,7 +5912,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>TECH_INGENIEUR_PROJETS_SPECIA</t>
+          <t>TECH_INGENIE</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -5945,7 +5946,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>RH_CHARGE_AFFAIRES_SOCIALES</t>
+          <t>RH_CHARGE_AF</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -5975,7 +5976,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>RH_CHARGE_FORMATION</t>
+          <t>RH_CHARGE_FO</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -6009,7 +6010,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>RH_CHARGE_GESTION_ADMINITRA</t>
+          <t>RH_CHARGE_GE</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -6039,7 +6040,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>RH_CHEF_PROJET_SIRH</t>
+          <t>RH_CHEF_PROJ</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -6069,7 +6070,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>RH_CHEF_EXP_FONCTION</t>
+          <t>RH_CHEF_EXP</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -6099,7 +6100,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>RH_CHEF_EXPLOITATION_CHARGE</t>
+          <t>RH_CHEF_EXPL</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -6129,7 +6130,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>RH_CHIEF_HUMAN_RESOURCES</t>
+          <t>RH_CHIEF_HUM</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -6159,7 +6160,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>RH_DIRECTEUR_ADJOINT_CHARGE</t>
+          <t>RH_DIRECTEUR</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -6189,7 +6190,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>RH_DIRECTRICE_ADJOINTE_RESS</t>
+          <t>RH_DIRECTRIC</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -6219,7 +6220,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>RH_RESPONSABLE_DEVELOPPEMEN</t>
+          <t>RH_RESPONSAB</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -6245,7 +6246,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>RH_RESPONSABLE_RSE_COORDINA</t>
+          <t>RH_RESPONSA2</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -6275,7 +6276,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>SUPP_AGENT_COURSES</t>
+          <t>SUPP_AGENT_C</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -6309,7 +6310,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>SUPP_CHARGE_BUREAU_ORDRE</t>
+          <t>SUPP_CHARGE</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -6339,7 +6340,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>SUPP_CHAUFFEUR</t>
+          <t>SUPP_CHAUFFE</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -6373,7 +6374,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>SUPP_OFFICE_MANAGER</t>
+          <t>SUPP_OFFICE</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -8903,7 +8904,7 @@
   <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="4" max="4"/>
   </cols>
@@ -8911,7 +8912,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Code (nécessite ALTER varchar(20), cf sql/alter_code_competence.sql)</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -22189,4 +22190,931 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Poste</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Colonne</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Longueur originale</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Limite colonne</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Texte original</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AUD_AUDITEUR / Auditeur Senior</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>559</v>
+      </c>
+      <c r="D2" t="n">
+        <v>250</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Evaluer et améliorer les mécanismes de gestion des risques, de controle et de gouvernance par le déploiement d'approches d'audit dynamiques et adaptives pour répondre aux évolutions sectorielles et réglementaires, assurant ainsi une couverture d'audit complète et pertinente. Maintenir l'objectivité et la rigueur de l'audit interne, tout en collaborant étroitement avec toutes les parties prenantes pour conseiller l'entreprise et renforcer sa capacité à anticiper et gérer les risques internes et externes, consolidant ainsi sa résilience organisationnelle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AUD_HEAD_OF / Head of Audit</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>567</v>
+      </c>
+      <c r="D3" t="n">
+        <v>250</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Evaluer et améliorer les mécanismes de gestion des risques, de contrôle et de gouvernance par le déploiement d'approches d'audit dynamiques et adaptives faces aux changements sectoriels et réglementaires afin de garantir une couverture d'audit complète et pertinente. Préserver l'objectivité, l'indépendance et la rigueur de l'audit interne, tout en collaborant étroitement avec toutes les parties prenantes pour conseiller l'entreprise et renforcer sa capacité à anticiper et gérer les risques internes et externes, consolidant ainsi sa résilience organisationnelle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DCM_CHARGEE / Chargée de la relation clients</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>259</v>
+      </c>
+      <c r="D4" t="n">
+        <v>250</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Agir en tant qu'interlocuteur privilégié des clients, en répondant efficacement à leurs besoins et en collaborant avec les différents départements de l'entreprise pour assurer une expérience client optimale, favorisant ainsi la fidélisation et la satisfaction</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DCM_CHEF_EX3 / Chef d'exploitation en charge CRC</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>271</v>
+      </c>
+      <c r="D5" t="n">
+        <v>250</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Gérer les aspects administratifs des ventes, en garantissant l'efficacité des opérations, la conformité des procédures et la satisfaction des clients, tout en collaborant étroitement avec les départements concernés pour atteindre les objectifs commerciaux de l'entreprise</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DCM_CHIEF_CO / Chief Commercial &amp; Marketing Officer</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>263</v>
+      </c>
+      <c r="D6" t="n">
+        <v>250</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Piloter les activités commerciales et marketing en alignant les objectifs stratégiques avec les opportunités du marché de l'acier, tout en optimisant les ressources et en développant les compétences des équipes pour atteindre une croissance durable et compétitive</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DCM_DIRECTE2 / Directeur Commercial Adjoint</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>265</v>
+      </c>
+      <c r="D7" t="n">
+        <v>250</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Assumer un rôle clé dans l'optimisation des performances commerciales en garantissant l'efficacité opérationnelle des équipes de vente, tout en veillant à l'harmonisation des actions avec les autres services pour atteindre les objectifs stratégiques de l'entreprise</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DCM_DIRECTE3 / Directeur des ventes</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>260</v>
+      </c>
+      <c r="D8" t="n">
+        <v>250</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Assumer la responsabilité de la performance commerciale de l'entreprise, en définissant et en exécutant des stratégies de vente efficaces, tout en optimisant les ressources humaines et financières pour maximiser la rentabilité et la compétitivité sur le marché</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DCM_RESPONS2 / Responsable administratif des ventes</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>271</v>
+      </c>
+      <c r="D9" t="n">
+        <v>250</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Gérer les aspects administratifs des ventes, en garantissant l'efficacité des opérations, la conformité des procédures et la satisfaction des clients, tout en collaborant étroitement avec les départements concernés pour atteindre les objectifs commerciaux de l'entreprise</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>FIN_CHARGE_C / Chargé Crédit Client</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>266</v>
+      </c>
+      <c r="D10" t="n">
+        <v>250</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Garant de la fiabilité des informations remontées (tableaux de bord, reportings, KPI)
+Garant du suivi des cautions bancaires (renouvellement, mobilisation)
+Garant des déclarations d'impayés à l'assurance dans les délais
+Garant du blocage d'un client sinistré sur SAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>FIN_CHEF_EXP / Chef d'Exploitation chargé du Contrôle de Gestion</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>OBSERVATIONS</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>558</v>
+      </c>
+      <c r="D11" t="n">
+        <v>550</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Intégrer la dimension QSEE dans le pilotage de l’activité, garantir au management une utilisation efficiente des ressources, assurer le respect des normes et exigences du contrôle interne, définir des objectifs alignés sur la stratégie de l’entreprise, animer un dispositif de pilotage favorisant leur atteinte, assurer le suivi et la revue périodique des targets ainsi que leur ajustement si nécessaire, inscrire la direction controlling dans une démarche d’amélioration continue et contribuer activement aux projets à forte valeur ajoutée pour l’entreprise</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>FIN_DIR_ADJ / Dir Adj controlling &amp; Cost Effectivness</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>INTER_INTERNE</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>272</v>
+      </c>
+      <c r="D12" t="n">
+        <v>250</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>100% du personnel de la Sonasid                                                                                          100% des Directions                                                                                                                  100% des retraités</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>FIN_DIRECTEU / Directeur Adjoint en charge de la trésorerie</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2303</v>
+      </c>
+      <c r="D13" t="n">
+        <v>250</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Garant de la performance cash (free cash flow)                                                                                                                                                                                                                                                                                                                                                                                                    Preserver la solvabilité et prévenir la cessation de paiement                                                                                                                                                                                                                                                                                           Garantir les financements                                                                                                                                                                                                                                                                                                                                       Optimiser la gestion des liquidités                                                                                                                                                                                                                                                                                                                                                    Support au business                                                                                                                                                                                                                                                                                                                                                                                Automatisation des process                                                                                                                                                                                                                                                                                                                                                                    Gestion des risques de change</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>FIN_DIRECTE3 / Directeur Comptabilité et Consolidation groupe Sonasid &amp; NSI</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>INTER_INTERNE</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>272</v>
+      </c>
+      <c r="D14" t="n">
+        <v>250</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>100% du personnel de la Sonasid                                                                                          100% des Directions                                                                                                                  100% des retraités</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>FIN_RESPONS4 / Responsable Reporting IFRS et amélioration continue du processus comptabilité du groupe Sonasid</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>INTITULE</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>95</v>
+      </c>
+      <c r="D15" t="n">
+        <v>90</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Responsable Reporting IFRS et amélioration continue du processus comptabilité du groupe Sonasid</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>DG_CHIEF_STR / Chief Strategy, Digital Officer &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>258</v>
+      </c>
+      <c r="D16" t="n">
+        <v>250</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Définir et mettre en œuvre les stratégies de l'entreprise, des systèmes d'information et de la gestion efficace de la chaîne d'approvisionnement pour garantir le fonctionnement optimal de l'aciérie, tout en répondant aux défis actuels et futurs de la Sonasid</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>IPP_TECH_202 / Ingénieur Projets Diplôme   Génie Procédés de l’EMI &amp; Master 2 en « Transition Énergétique » de l’École des Ponts ParisTech</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>INTITULE</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>123</v>
+      </c>
+      <c r="D17" t="n">
+        <v>90</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Ingénieur Projets Diplôme   Génie Procédés de l’EMI &amp; Master 2 en « Transition Énergétique » de l’École des Ponts ParisTech</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>GEN_CHARGE_T / Chargé de Transport</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>INTER_INTERNE</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>376</v>
+      </c>
+      <c r="D18" t="n">
+        <v>250</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Direction finance                                                                                                                                                                                                                                                                                                                                                  Direction commerciale</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>GEN_CHARGE_T / Chargé de Transport</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>RESULTAT_ATTENDU</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>359</v>
+      </c>
+      <c r="D19" t="n">
+        <v>250</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Taux de conformité aux normes de sécurité                                                                                                                                                                                                                                                                                              Temps de traitement des factures</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>GEN_CHARGE_C / Chargé de consignation</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>RESULTAT_ATTENDU</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>759</v>
+      </c>
+      <c r="D20" t="n">
+        <v>250</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Taux de conformité aux réglementations                                                                                                                                                                                                                                                                                                                                           Taux de disponibilité  des PF au niveau des sites de consignation                                                                                                                                                                                                                                                                           Taux de rotation des stocks dans les sites de consignation</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>GEN_DIRECTRI / Directrice Adjointe en charge de la Supply Chain</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>INTER_INTERNE</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>384</v>
+      </c>
+      <c r="D21" t="n">
+        <v>250</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>- Direction industrielle
+- Direction commerciale
+- Direction achat                                                                                                                                                                                                                                                                       - Autres directions du support (Finance, Qualité, SQEE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>GEN_DIRECTRI / Directrice Adjointe en charge de la Supply Chain</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>RESULTAT_ATTENDU</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1048</v>
+      </c>
+      <c r="D22" t="n">
+        <v>250</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Taux de conformité aux normes de sécurité et environnementales                                                                                                                                                                                                                                                                      '- Temps de séjour camions.                                                                                                                                                                                                                                                                                                                                             '- Fiabilité des stocks: zero écart de stock                                                                                                                                                                                                                                                                                      '- Taux de réalisation réalisé vs planifié</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>GEN_INGENIEU / Ingénieur SST</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>INTER_INTERNE</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>380</v>
+      </c>
+      <c r="D23" t="n">
+        <v>250</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>- Direction industrielle                                                                                                                                                                                                                                                                                                                                               Direction commerciale</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>GEN_RESPONS2 / Responsable Opérations Logistiques Import / Export</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>282</v>
+      </c>
+      <c r="D24" t="n">
+        <v>250</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Rationaliser les processus logistiques internationaux pour assurer la fluidité des échanges, réduire les coûts, les délais et les risques et garantir une gestion transparente des mouvements de marchandises, tout en respectant les réglementations douanières et les normes de sécurité</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>GEN_RESPONS2 / Responsable Opérations Logistiques Import / Export</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>INTER_INTERNE</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>384</v>
+      </c>
+      <c r="D25" t="n">
+        <v>250</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>- Direction industrielle
+- Direction commerciale
+- Direction achat                                                                                                                                                                                                                                                                       - Autres directions du support (Finance, Qualité, SQEE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>GEN_RESPONS2 / Responsable Opérations Logistiques Import / Export</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>RESULTAT_ATTENDU</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>340</v>
+      </c>
+      <c r="D26" t="n">
+        <v>250</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Taux de conformité aux normes de sécurité et environnementales                                                                                                                                                                                                                                                  '- Temps de traitement des commandes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>GEN_RESPONS4 / Responsable Sonasid Distribution</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>RESULTAT_ATTENDU</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>742</v>
+      </c>
+      <c r="D27" t="n">
+        <v>250</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Taux de conformité aux normes de sécurité                                                                                                                                                                                                                                                                                                    Fiabilité des stocks  : zéro écart de stock                                                                                                                                                                                                                                                                                                                               Taux de conformité aux normes de qualité des PF</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>GEN_RESPONS5 / Responsable Transport</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>RESULTAT_ATTENDU</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1045</v>
+      </c>
+      <c r="D28" t="n">
+        <v>250</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Taux de conformité aux normes de sécurité                                                                                                                                                                                                                                                                                                         Taux de remplissage camions                                                                                                                                                                                                                                                                                                                          Taux d'utilisation optimale des flottes de véhicules                                                                                                                                                                                                                                                                                         Temps de traitement des commandes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>GEN_RESPONS6 / Responsable des activités portuaires</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>295</v>
+      </c>
+      <c r="D29" t="n">
+        <v>250</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Coordonner les activités portuaires pour assurer la qualité du service, la réduction des coûts, le respect des normes de sécurité et environnementales, et l'efficacité des opérations de chargement et de déchargement, tout en maintenant des relations solides avec les parties prenantes portuaires</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>GEN_RESPONS6 / Responsable des activités portuaires</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>RESULTAT_ATTENDU</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>643</v>
+      </c>
+      <c r="D30" t="n">
+        <v>250</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Taux de conformité aux normes de sécurité et environnementales                                                                                                                                                                                                                                                - Nombre de rotation camions                                                                                                                                                                                                                                                                                             -Volume transféré port usine</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>GEN_SUPERVI2 / Superviseur pont Bascule</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>290</v>
+      </c>
+      <c r="D31" t="n">
+        <v>250</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Assurer la fiabilité des données de pesage et l’optimisation des opérations logistiques en supervisant les activités du pont bascule et en maintenant une communication fluide avec les équipes internes et externes pour prévenir les anomalies et garantir la satisfaction des parties prenantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>GEN_SUPPLY_C / Supply Chain Manager</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>293</v>
+      </c>
+      <c r="D32" t="n">
+        <v>250</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Coordonner les activités logistiques opérationnelles, y compris l'approvisionnement, le stockage et la distribution, afin d'optimiser les coûts, d'améliorer la performance et de garantir la satisfaction des clients internes et externes dans le cadre des directives stratégiques de l'entreprise</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>GEN_SUPPLY_C / Supply Chain Manager</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>RESULTAT_ATTENDU</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>743</v>
+      </c>
+      <c r="D33" t="n">
+        <v>250</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Taux de satisfaction des clients internes et externes et prestataires (impayés)                                                                                                                                                                                                                                                                                      Taux de réalisation de production  planifié vs réalisé                                                                                                                                                                                                                                                                                                                Taux de remplissage camions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>RH_CHARGE_FO / Chargé de Formation</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>322</v>
+      </c>
+      <c r="D34" t="n">
+        <v>250</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Le déploiement du périmètre du poste a un impact direct sur la déroulement efficace du plan de formation de Sonasid : Garantir la coordination et l’exécution efficace des actions de formation pour assurer le développement des compétences des collaborateurs, tout en respectant les objectifs du plan de formation de Sonasid</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>RH_CHEF_PROJ / Chef de projet SIRH</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>347</v>
+      </c>
+      <c r="D35" t="n">
+        <v>250</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Le déploiement du périmètre du poste a un impact direct sur la disponibilité d'outils performants pour une gestion RH de proximité : Garantir la mise en œuvre de solutions SIRH performantes, adaptées aux besoins des utilisateurs, tout en assurant la sécurité et l’intégrité des données, pour améliorer l’efficacité et la proximité de la gestion RH</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>RH_CHEF_EXPL / Chef d’exploitation en charge des Projets RH</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>334</v>
+      </c>
+      <c r="D36" t="n">
+        <v>250</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Le déploiement du périmètre du poste a un impact direct sur la structuration et l'optimisation des processus RH : Garantir la mise en œuvre efficace des projets de développement RH pour structurer et optimiser les processus, tout en répondant aux besoins stratégiques du business et en alignement avec la feuille de route RH du groupe</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>RH_CHIEF_HUM / Chief Human Resources &amp; CSR</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>383</v>
+      </c>
+      <c r="D37" t="n">
+        <v>250</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Le déploiement du périmètre du poste a un impact direct sur la culture d'entreprise, la réputation sociale et le bien-être des employés : Assurer un leadership stratégique pour renforcer la culture d’entreprise, promouvoir la durabilité et l’éthique, et optimiser l’engagement des collaborateurs tout en soutenant la réputation sociale de Sonasid et son impact positif sur la société</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>RH_DIRECTEUR / Directeur Adjoint en charge du développement RH</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>490</v>
+      </c>
+      <c r="D38" t="n">
+        <v>250</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Le déploiement du périmètre du poste a un impact direct sur la cohésion entre les besoins en compétences de l'entreprise et les attentes individuels des collaborateurs en matière d'employabilité et de gestion des carrières : Piloter les initiatives stratégiques de formation, de gestion des talents et de développement organisationnel pour aligner les compétences des collaborateurs sur les besoins de l’entreprise, tout en renforçant leur employabilité et leur satisfaction professionnelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>RH_RESPONSA2 / Responsable RSE et coordinatrice ESG</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>DIMENSION</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>397</v>
+      </c>
+      <c r="D39" t="n">
+        <v>250</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Le poste joue un rôle crucial dans la consolidation de la réputation sociétale et environnementale de Sonasid, en veillant à ce que les activités de l’entreprise soient perçues comme éthiques et durables. Il s’agit également de maximiser l’impact des initiatives RSE sur le positionnement stratégique global de l’entreprise tout en répondant aux attentes des parties prenantes internes et externes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>